<commit_message>
little edited in opi khola and jcb log and checked nirmal lawaju etabs
</commit_message>
<xml_diff>
--- a/2083_2084/estimate/budget maag estimate/dashain baato sarsafai/jcb log book - Copy.xlsx
+++ b/2083_2084/estimate/budget maag estimate/dashain baato sarsafai/jcb log book - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\2083_2084\estimate\budget maag estimate\dashain baato sarsafai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A452371-8416-4DFF-AE27-57C27E5015A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34750F2E-5397-47A9-A285-0ADA03F610DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="43">
   <si>
     <t>सि. न</t>
   </si>
@@ -199,6 +199,9 @@
   </si>
   <si>
     <t>khadka gaun, bhumedanda</t>
+  </si>
+  <si>
+    <t>rainfall and no work</t>
   </si>
 </sst>
 </file>
@@ -332,7 +335,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -409,6 +412,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -423,19 +435,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -729,28 +728,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" x14ac:dyDescent="0.9">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="2" spans="1:4" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
     </row>
     <row r="3" spans="1:4" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
     </row>
     <row r="4" spans="1:4" ht="30.75" x14ac:dyDescent="0.75">
       <c r="A4" s="14"/>
@@ -759,12 +758,12 @@
       <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.75">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
     </row>
     <row r="6" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="1.3">
       <c r="A6" s="4" t="s">
@@ -988,34 +987,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" x14ac:dyDescent="0.9">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
     </row>
     <row r="4" spans="1:6" ht="30.75" x14ac:dyDescent="0.75">
       <c r="A4" s="14"/>
@@ -1026,14 +1025,14 @@
       <c r="F4" s="14"/>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.75">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.75">
       <c r="A6" s="23"/>
@@ -1080,24 +1079,24 @@
       <c r="F9" s="28"/>
     </row>
     <row r="10" spans="1:6" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A11" s="34"/>
-      <c r="B11" s="34"/>
+      <c r="A11" s="37"/>
+      <c r="B11" s="37"/>
       <c r="C11" s="7" t="s">
         <v>31</v>
       </c>
@@ -1107,7 +1106,7 @@
       <c r="E11" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="34"/>
+      <c r="F11" s="37"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.6">
       <c r="A12" s="25">
@@ -1126,7 +1125,7 @@
         <f>D12-C12</f>
         <v>10.100000000000364</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="30">
         <v>46310</v>
       </c>
     </row>
@@ -1145,10 +1144,10 @@
         <v>9919.1</v>
       </c>
       <c r="E13" s="8">
-        <f t="shared" ref="E13:E16" si="0">D13-C13</f>
+        <f t="shared" ref="E13:E17" si="0">D13-C13</f>
         <v>7.3999999999996362</v>
       </c>
-      <c r="F13" s="35">
+      <c r="F13" s="30">
         <v>46311</v>
       </c>
     </row>
@@ -1170,7 +1169,7 @@
         <f t="shared" si="0"/>
         <v>10.699999999998909</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="30">
         <v>46321</v>
       </c>
     </row>
@@ -1192,7 +1191,7 @@
         <f t="shared" si="0"/>
         <v>11.600000000000364</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="30">
         <v>46322</v>
       </c>
     </row>
@@ -1214,7 +1213,7 @@
         <f t="shared" si="0"/>
         <v>10.600000000000364</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="30">
         <v>46323</v>
       </c>
     </row>
@@ -1229,9 +1228,14 @@
         <f t="shared" si="1"/>
         <v>9952</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="35">
+      <c r="D17" s="11">
+        <v>9962.7000000000007</v>
+      </c>
+      <c r="E17" s="11">
+        <f t="shared" si="0"/>
+        <v>10.700000000000728</v>
+      </c>
+      <c r="F17" s="30">
         <v>46324</v>
       </c>
     </row>
@@ -1239,14 +1243,18 @@
       <c r="A18" s="25">
         <v>7</v>
       </c>
-      <c r="B18" s="9"/>
+      <c r="B18" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="C18" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>9962.7000000000007</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
+      <c r="F18" s="30">
+        <v>46325</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.6">
       <c r="A19" s="25">
@@ -1402,36 +1410,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" x14ac:dyDescent="0.9">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
       <c r="G1" s="24"/>
     </row>
     <row r="2" spans="1:7" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
       <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:7" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
       <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" ht="30.75" x14ac:dyDescent="0.75">
@@ -1444,14 +1452,14 @@
       <c r="G4" s="14"/>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.75">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
       <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.75">
@@ -1503,25 +1511,25 @@
       <c r="G9" s="28"/>
     </row>
     <row r="10" spans="1:7" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="G10" s="36"/>
+      <c r="G10" s="31"/>
     </row>
     <row r="11" spans="1:7" ht="30.75" x14ac:dyDescent="0.75">
-      <c r="A11" s="34"/>
-      <c r="B11" s="34"/>
+      <c r="A11" s="37"/>
+      <c r="B11" s="37"/>
       <c r="C11" s="7" t="s">
         <v>31</v>
       </c>
@@ -1531,8 +1539,8 @@
       <c r="E11" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="36"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="31"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A12" s="25">
@@ -1551,10 +1559,10 @@
         <f>D12-C12</f>
         <v>12</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="30">
         <v>46321</v>
       </c>
-      <c r="G12" s="37"/>
+      <c r="G12" s="32"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A13" s="25">
@@ -1574,10 +1582,10 @@
         <f>D13-C13</f>
         <v>10.400000000000091</v>
       </c>
-      <c r="F13" s="35">
+      <c r="F13" s="30">
         <v>46322</v>
       </c>
-      <c r="G13" s="37"/>
+      <c r="G13" s="32"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A14" s="25">
@@ -1597,10 +1605,10 @@
         <f>D14-C14</f>
         <v>11.099999999999909</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="30">
         <v>46323</v>
       </c>
-      <c r="G14" s="37"/>
+      <c r="G14" s="32"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A15" s="25">
@@ -1613,23 +1621,31 @@
         <f>D14</f>
         <v>1558.1</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="35">
+      <c r="D15" s="11">
+        <v>1566.8</v>
+      </c>
+      <c r="E15" s="11">
+        <f>D15-C15</f>
+        <v>8.7000000000000455</v>
+      </c>
+      <c r="F15" s="30">
         <v>46324</v>
       </c>
-      <c r="G15" s="37"/>
+      <c r="G15" s="32"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A16" s="25">
         <v>5</v>
       </c>
-      <c r="B16" s="9"/>
+      <c r="B16" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="38"/>
+      <c r="F16" s="30">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A17" s="25">
@@ -1640,7 +1656,6 @@
       <c r="D17" s="20"/>
       <c r="E17" s="20"/>
       <c r="F17" s="20"/>
-      <c r="G17" s="38"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A18" s="25">
@@ -1651,7 +1666,7 @@
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
       <c r="F18" s="11"/>
-      <c r="G18" s="39"/>
+      <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.6">
       <c r="A19" s="25">
@@ -1662,7 +1677,7 @@
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
-      <c r="G19" s="39"/>
+      <c r="G19" s="13"/>
     </row>
     <row r="20" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="12"/>

</xml_diff>